<commit_message>
Extend the rate history to 2023 and add Supertasas and ISR history
</commit_message>
<xml_diff>
--- a/sofipo_savings.xlsx
+++ b/sofipo_savings.xlsx
@@ -138,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="institutions" displayName="institutions" ref="A1:H14" headerRowCount="1">
-  <autoFilter ref="A1:H14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="institutions" displayName="institutions" ref="A1:H15" headerRowCount="1">
+  <autoFilter ref="A1:H15"/>
   <tableColumns count="8">
     <tableColumn id="1" name="institution"/>
     <tableColumn id="2" name="type"/>
@@ -251,8 +251,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="rates_history" displayName="rates_history" ref="A1:K97" headerRowCount="1">
-  <autoFilter ref="A1:K97"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="rates_history" displayName="rates_history" ref="A1:K147" headerRowCount="1">
+  <autoFilter ref="A1:K147"/>
   <tableColumns count="11">
     <tableColumn id="1" name="date"/>
     <tableColumn id="2" name="institution"/>
@@ -296,8 +296,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tax_params" displayName="tax_params" ref="A1:G12" headerRowCount="1">
-  <autoFilter ref="A1:G12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tax_params" displayName="tax_params" ref="A1:G17" headerRowCount="1">
+  <autoFilter ref="A1:G17"/>
   <tableColumns count="7">
     <tableColumn id="1" name="param"/>
     <tableColumn id="2" name="value"/>
@@ -663,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1173,35 +1173,75 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Supertasas</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SOFIPO</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prosofipo</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>220596.6</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Covered only through the Germán Mi Amigo Dinero video series (rate history only, no current product). Mostly fixed terms.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@miamigodinero</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>video only</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>CETES (via GBM or Cetesdirecto)</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Federal government</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Government debt, no deposit insurance needed. Buying through GBM may add fees (not modeled). Withholding assumed at the 0.90% rate.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://www.tasas.mx/</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>rates yes; GBM fees unverified</t>
         </is>
@@ -29331,7 +29371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32198,202 +32238,190 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>2023-03-02</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Fixed terms, 11-13% by term; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en cada plazo? (Marzo 2023), 2023-03-02, https://www.youtube.com/watch?v=gmy1pM3RSQY</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Nu</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Cajita (on demand)</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
-        <v>0</v>
-      </c>
-      <c r="E68" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>https://www.nmas.com.mx/economia/finanzas-personales/nu-ya-es-un-banco-en-mexico-esto-significa-para-cuentahabientes-y-que-cambia-en-2026/</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>2023-04-02</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Fixed terms, 10-11%; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ABRIL 2023? CETES, SOFIPOS, Hey Banco, mercado pago, etc., 2023-04-02, https://www.youtube.com/watch?v=qABJs5rFw7A</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Nu</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Cajita Turbo</t>
-        </is>
-      </c>
-      <c r="D69" t="n">
-        <v>0</v>
-      </c>
-      <c r="E69" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F69" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G69" t="n">
-        <v>0.065</v>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>Monthly debit card purchase</t>
-        </is>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>https://www.nmas.com.mx/economia/finanzas-personales/nu-ya-es-un-banco-en-mexico-esto-significa-para-cuentahabientes-y-que-cambia-en-2026/</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>2023-06-02</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en JUNIO 2023? CETES, SOFIPOS, Hey Banco, KLAR, etc., 2023-06-02, https://www.youtube.com/watch?v=mx8pE7Ohydk</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Nu</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Fixed term 7d</t>
-        </is>
-      </c>
-      <c r="D70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E70" t="n">
-        <v>0.0655</v>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/institucion/nu</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>2023-08-03</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Fixed term; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, CETES detienen su caída! - ¿Quién PAGA MÁS en Agosto 2023?, 2023-08-03, https://www.youtube.com/watch?v=0UVRneDYElU</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Nu</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Fixed term 180d</t>
-        </is>
-      </c>
-      <c r="D71" t="n">
-        <v>180</v>
-      </c>
-      <c r="E71" t="n">
-        <v>0.068</v>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/institucion/nu</t>
-        </is>
-      </c>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2023-11-03</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ualá</t>
+          <t>Finsus</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>On demand (Plus)</t>
-        </is>
-      </c>
-      <c r="D72" t="n">
-        <v>0</v>
+          <t>Headline rate (video)</t>
+        </is>
       </c>
       <c r="E72" t="n">
         <v>0.15</v>
       </c>
-      <c r="F72" t="n">
-        <v>30000</v>
-      </c>
-      <c r="G72" t="n">
-        <v>0.0675</v>
-      </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Plus level; base account about 6.75%</t>
+          <t>Fixed term; term not stated in video</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>https://www.rendimientosmexico.com/instrumentos/uala</t>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en noviembre 2023? - Opciones con 15% de rendimiento, 200% más ISR, 2023-11-03, https://www.youtube.com/watch?v=_JHrncIaD2k</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -32403,89 +32431,80 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>2023-11-03</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>0</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>No cap, no conditions; start of the 15% rate war</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en noviembre 2023? - Opciones con 15% de rendimiento, 200% más ISR, 2023-11-03, https://www.youtube.com/watch?v=_JHrncIaD2k</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Klar</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>On demand (Plus/Platino)</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
-        <v>0</v>
-      </c>
-      <c r="E73" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>Regular balance; 6% standard. The 15% is the separate Inversión Max product</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/institucion/klar</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2024-01-03</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Klar</t>
+          <t>Nu</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Inversión Max (Plus/Platino)</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>0</v>
+          <t>Headline rate (video)</t>
+        </is>
       </c>
       <c r="E74" t="n">
         <v>0.15</v>
       </c>
-      <c r="F74" t="n">
-        <v>25000</v>
-      </c>
-      <c r="G74" t="n">
-        <v>0.08</v>
-      </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>2,500 monthly spend; cap from video (Dec 2025)</t>
+          <t>term not stated in video; Nu was a SOFIPO at this date</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>https://deceroalinfinito.com/mejores-sofipos</t>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ENERO 2024? - CETES y FINAMEX bajan, 2024-01-03, https://www.youtube.com/watch?v=JWT4v1Y1v9A</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -32495,213 +32514,201 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>yes (cap from video)</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>2024-02-02</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Klar rises a lot this month</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en FEBRERO 2024? - Cajitas en NU, KLAR sube mucho, DINN baja tasa, 2024-02-02, https://www.youtube.com/watch?v=4t6Kf4HouwU</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Klar</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Fixed term 365d (Plus/Platino)</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>365</v>
-      </c>
-      <c r="E75" t="n">
-        <v>0.08500000000000001</v>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>Plus/Platino</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/institucion/klar</t>
-        </is>
-      </c>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>2024-02-02</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Supertasas</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Mostly fixed terms; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en FEBRERO 2024? - Cajitas en NU, KLAR sube mucho, DINN baja tasa, 2024-02-02, https://www.youtube.com/watch?v=4t6Kf4HouwU</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Banco Plata</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Ahorro Flexible (base)</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>0</v>
-      </c>
-      <c r="E76" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
-        </is>
-      </c>
-      <c r="J76" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>2024-03-02</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Cajita (on demand)</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Cajitas launched Feb 2024; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en MARZO 2024? - CETES bajan, Finsus sube a 16%, ¿Banxico bajará?, 2024-03-02, https://www.youtube.com/watch?v=eFXqSq8hqS8</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Banco Plata</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Ahorro Flexible (Plata+)</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>99 MXN + IVA monthly; cut from 10% in Aug 2026</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
-        </is>
-      </c>
-      <c r="J77" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>2024-03-02</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>0</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en MARZO 2024? - CETES bajan, Finsus sube a 16%, ¿Banxico bajará?, 2024-03-02, https://www.youtube.com/watch?v=eFXqSq8hqS8</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Banco Plata</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Fixed term 360d (Plata+)</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>365</v>
-      </c>
-      <c r="E78" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>Plata+; base terms 7-8%</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
-        </is>
-      </c>
-      <c r="J78" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>secondary</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2024-03-02</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Openbank</t>
+          <t>Finsus</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Apartados Open</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>0</v>
+          <t>Headline rate (video)</t>
+        </is>
       </c>
       <c r="E79" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F79" t="n">
-        <v>30000</v>
-      </c>
-      <c r="G79" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Open+ debit account; 6.5% above 1M</t>
+          <t>Long fixed terms; term not stated in video</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>https://www.tasas.mx/institucion/openbank</t>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en MARZO 2024? - CETES bajan, Finsus sube a 16%, ¿Banxico bajará?, 2024-03-02, https://www.youtube.com/watch?v=eFXqSq8hqS8</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -32711,89 +32718,80 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>conflict (see institutions)</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>2024-04-02</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Cajita (on demand)</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ABRIL 2024? - CAÍDAS por todos lados, 2024-04-02, https://www.youtube.com/watch?v=axxIJ237U9s</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Mercado Pago</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>On demand (no Meli+)</t>
-        </is>
-      </c>
-      <c r="D80" t="n">
-        <v>0</v>
-      </c>
-      <c r="E80" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="F80" t="n">
-        <v>25000</v>
-      </c>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>Without subscription</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/institucion/mercadopago</t>
-        </is>
-      </c>
-      <c r="J80" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2024-04-02</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>DiDi</t>
+          <t>Finsus</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>On demand</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>0</v>
+          <t>Headline rate (video)</t>
+        </is>
       </c>
       <c r="E81" t="n">
         <v>0.15</v>
       </c>
-      <c r="F81" t="n">
-        <v>10000</v>
-      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Rate on balance above 10,000 not found</t>
+          <t>Fixed term; term not stated in video</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>https://www.tasas.mx/</t>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ABRIL 2024? - CAÍDAS por todos lados, 2024-04-02, https://www.youtube.com/watch?v=axxIJ237U9s</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -32803,623 +32801,2734 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>yes (excess rate unverified)</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>2024-05-02</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en MAYO 2024? - SIGUEN LAS CAÍDAS, 2024-05-02, https://www.youtube.com/watch?v=D92SpdExA9k</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Stori</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>On demand</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>0</v>
-      </c>
-      <c r="E82" t="n">
-        <v>0.0725</v>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>https://deceroalinfinito.com/mejores-sofipos</t>
-        </is>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>2024-08-03</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>term not stated in video; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en AGOSTO 2024? - Los CETES quedan a deber, 2024-08-03, https://www.youtube.com/watch?v=pNDU4jQxVac</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Stori</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Fixed term 30d</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>30</v>
-      </c>
-      <c r="E83" t="n">
-        <v>0.07049999999999999</v>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>2024-08-03</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en AGOSTO 2024? - Los CETES quedan a deber, 2024-08-03, https://www.youtube.com/watch?v=pNDU4jQxVac</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Stori</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Fixed term 90d</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>90</v>
-      </c>
-      <c r="E84" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
+          <t>2024-10-03</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Stori adds fixed terms this month; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en OCTUBRE 2024? - NU baja tasas, meli dólar llega, stori tiene plazos, 2024-10-03, https://www.youtube.com/watch?v=Ju5oYtKpAKo</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Stori</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Fixed term 180d</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>180</v>
-      </c>
-      <c r="E85" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J85" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>2025-01-04</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Depends on account level</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ENERO 2025? - CETES recupera el 10%, NU baja tasas, KLAR cambia mucho, 2025-01-04, https://www.youtube.com/watch?v=3nRL92xKGy0</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Stori</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Fixed term 365d</t>
-        </is>
-      </c>
-      <c r="D86" t="n">
-        <v>365</v>
-      </c>
-      <c r="E86" t="n">
-        <v>0.0825</v>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J86" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>2025-02-04</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Fixed term; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en FEBRERO 2025? - NU domina, ARANCELES, y constancias de impuestos, 2025-02-04, https://www.youtube.com/watch?v=Om-l5Akl7to</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Finsus</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>On demand</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E87" t="n">
-        <v>0.0701</v>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>https://deceroalinfinito.com/mejores-sofipos</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>2025-04-03</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>term not stated in video; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ABRIL 2025? - CETES CAEN, Now Bank es nueva opción, NU cambia de tasa pronto, 2025-04-03, https://www.youtube.com/watch?v=l7D2bz8tBtg</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Finsus</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Fixed term 30d</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
-        <v>30</v>
-      </c>
-      <c r="E88" t="n">
-        <v>0.07190000000000001</v>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
+          <t>2025-05-03</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>9-15% depending on product and cap; term not stated in video; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en MAYO 2025? - SOFIPO quiebra, mercado pago baja, NU será banco, 2025-05-03, https://www.youtube.com/watch?v=AH2vQLe0dQQ</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Finsus</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Fixed term 90d</t>
-        </is>
-      </c>
-      <c r="D89" t="n">
-        <v>90</v>
-      </c>
-      <c r="E89" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>DiDi</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Announced: DiDi to pay 15%</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en JUNIO 2025? - DIDI dará 15%, Novedades en NU, KLAR baja tasas, 2025-06-05, https://www.youtube.com/watch?v=w1QWl47g0uc</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Finsus</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Fixed term 180d</t>
-        </is>
-      </c>
-      <c r="D90" t="n">
-        <v>180</v>
-      </c>
-      <c r="E90" t="n">
-        <v>0.0759</v>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>12-14%, capped; term not stated in video; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en JULIO 2025? - Cashback en NU+, 16% en ualá, didi al 15%, 2025-07-03, https://www.youtube.com/watch?v=3qbfW5NrZog</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Finsus</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>Fixed term 365d</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
-        <v>365</v>
-      </c>
-      <c r="E91" t="n">
-        <v>0.08690000000000001</v>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Fixed term; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en JULIO 2025? - Cashback en NU+, 16% en ualá, didi al 15%, 2025-07-03, https://www.youtube.com/watch?v=3qbfW5NrZog</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Kubo Financiero</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Fixed term 90d</t>
-        </is>
-      </c>
-      <c r="D92" t="n">
-        <v>90</v>
-      </c>
-      <c r="E92" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>Withdrawal problems reported May-Jun 2026</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>2025-07-03</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en JULIO 2025? - Cashback en NU+, 16% en ualá, didi al 15%, 2025-07-03, https://www.youtube.com/watch?v=3qbfW5NrZog</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Kubo Financiero</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Fixed term 365d</t>
-        </is>
-      </c>
-      <c r="D93" t="n">
-        <v>365</v>
-      </c>
-      <c r="E93" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>Withdrawal problems reported May-Jun 2026</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>2025-08-05</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Sharp drop; term not stated in video; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en AGOSTO 2025? - DESPLOME en NU, Stori, KLAR, los CETES se recuperan, 2025-08-05, https://www.youtube.com/watch?v=w8--F9sqbVw</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>CETES (via GBM or Cetesdirecto)</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>CETES 28d</t>
-        </is>
-      </c>
-      <c r="D94" t="n">
-        <v>28</v>
-      </c>
-      <c r="E94" t="n">
-        <v>0.0615</v>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>2025-08-05</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Sharp drop; base level</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en AGOSTO 2025? - DESPLOME en NU, Stori, KLAR, los CETES se recuperan, 2025-08-05, https://www.youtube.com/watch?v=w8--F9sqbVw</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>CETES (via GBM or Cetesdirecto)</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>CETES 91d</t>
-        </is>
-      </c>
-      <c r="D95" t="n">
-        <v>91</v>
-      </c>
-      <c r="E95" t="n">
-        <v>0.0659</v>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>2025-10-04</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en OCTUBRE 2025?, 2025-10-04, https://www.youtube.com/watch?v=7jNCqK43Fkc</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>CETES (via GBM or Cetesdirecto)</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>CETES 182d</t>
-        </is>
-      </c>
-      <c r="D96" t="n">
-        <v>182</v>
-      </c>
-      <c r="E96" t="n">
-        <v>0.06909999999999999</v>
-      </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>https://www.tasas.mx/</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
+          <t>2025-10-04</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>5-12.5% across products; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en OCTUBRE 2025?, 2025-10-04, https://www.youtube.com/watch?v=7jNCqK43Fkc</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>8-9%; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en NOVIEMBRE 2025?, 2025-11-04, https://www.youtube.com/watch?v=FYmxm2lTYvQ</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en NOVIEMBRE 2025?, 2025-11-04, https://www.youtube.com/watch?v=FYmxm2lTYvQ</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Stori rises a lot; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en DICIEMBRE 2025?, 2025-12-03, https://www.youtube.com/watch?v=-rDq0PLHGs4</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2025-12-03</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>0.135</v>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en DICIEMBRE 2025?, 2025-12-03, https://www.youtube.com/watch?v=-rDq0PLHGs4</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Cajita (on demand)</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>0</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Nu cuts; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ENERO 2026?, 2026-01-07, https://www.youtube.com/watch?v=zOLucpISr7c</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en ENERO 2026?, 2026-01-07, https://www.youtube.com/watch?v=zOLucpISr7c</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-02-04</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>0.1325</v>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>term not stated in video</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, ¿Quién PAGA MÁS en FEBRERO 2026?, 2026-02-04, https://www.youtube.com/watch?v=tqd4ME8JhSM</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Supertasas</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>7.0-7.6% mentioned; mostly fixed terms; term not stated in video</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, NU ya se RINDIÓ, aquí GANAS MÁS, 2026-04-09, https://www.youtube.com/watch?v=ivm1_uAzvuY</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Fixed term 90d</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>90</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>No requirement</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Las Tasas Cambiaron... Junio, 2026-06-04, https://www.youtube.com/watch?v=4-ZB5rI_WnA</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Cajita Turbo</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Capped (amount not stated) with an activation condition; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Adiós Revolut: Se nos Cayó un Grande!, 2026-06-24, https://www.youtube.com/watch?v=XTDcKIUcak4</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Cajita Turbo</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Capped (amount not stated) with an activation condition; Nu was a SOFIPO at this date</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Revolut se Rindió. Estas son las Alternativas., 2026-07-02, https://www.youtube.com/watch?v=UurM0cORmNI</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>0</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F109" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>About 3,000 MXN monthly deposits; cut to 12% this month</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Las Tasas Cambiaron... Julio, 2026-07-05, https://www.youtube.com/watch?v=YcVJv9_32r4</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Cajita Turbo</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>No cap</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, KUBO Lanza una "Cajita Turbo" SIN TOPE!!, 2026-07-11, https://www.youtube.com/watch?v=ABZytAfldQk</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>DiDi</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F111" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Excess about 7.5%; about 12.3% blended at 15,000; paid daily</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Las Mejores Inversiones en 2026, Rankeadas, 2026-07-16, https://www.youtube.com/watch?v=U6m5NDabFec</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Fixed term 90d</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>90</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>No requirement</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Fue un ERROR Aceptar las Inversiones Topadas, 2026-07-30, https://www.youtube.com/watch?v=jzhrIrAru-E</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Fixed term 180d</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>180</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>No requirement</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Fue un ERROR Aceptar las Inversiones Topadas, 2026-07-30, https://www.youtube.com/watch?v=jzhrIrAru-E</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Fixed term 120d (membership)</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>120</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0.115</v>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Paid membership, about 500 MXN a year</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Las Tasas Cambiaron... Agosto 2026, 2026-08-07, https://www.youtube.com/watch?v=xoA6vk1q0Mo</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Cajita (on demand)</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Regular Cajitas; Nu a bank since 2026-08-06</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Cambios en las Cajitas NU Explicados, 2026-08-07, https://www.youtube.com/watch?v=pkGJ4boI6tk</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>DiDi</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>0</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F116" t="n">
+        <v>10000</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Excess about 7.5%</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, La Didi Cuenta Debería Preocuparnos, 2026-08-24, https://www.youtube.com/watch?v=FnZBsYYLf4k</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Headline rate (video)</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>13% tier tied to a 2,500 MXN requirement; terms got worse this month</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Germán Mi Amigo Dinero, Así Ganas $6,297.04 al Mes Sin Hacer Nada, 2026-09-17, https://www.youtube.com/watch?v=hvP_dB63NT8</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>video (auto-captions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Cajita (on demand)</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>0</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>https://www.nmas.com.mx/economia/finanzas-personales/nu-ya-es-un-banco-en-mexico-esto-significa-para-cuentahabientes-y-que-cambia-en-2026/</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Cajita Turbo</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>0</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F119" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Monthly debit card purchase</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>https://www.nmas.com.mx/economia/finanzas-personales/nu-ya-es-un-banco-en-mexico-esto-significa-para-cuentahabientes-y-que-cambia-en-2026/</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Fixed term 7d</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>7</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0.0655</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/nu</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Nu</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Fixed term 180d</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>180</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0.068</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/nu</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Ualá</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>On demand (Plus)</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>0</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F122" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0.0675</v>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Plus level; base account about 6.75%</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>https://www.rendimientosmexico.com/instrumentos/uala</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>On demand (Plus/Platino)</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>0</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Regular balance; 6% standard. The 15% is the separate Inversión Max product</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/klar</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Inversión Max (Plus/Platino)</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F124" t="n">
+        <v>25000</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>2,500 monthly spend; cap from video (Dec 2025)</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>https://deceroalinfinito.com/mejores-sofipos</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>yes (cap from video)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Klar</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Fixed term 365d (Plus/Platino)</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>365</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Plus/Platino</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/klar</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Banco Plata</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Ahorro Flexible (base)</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Banco Plata</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Ahorro Flexible (Plata+)</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>99 MXN + IVA monthly; cut from 10% in Aug 2026</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Banco Plata</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Fixed term 360d (Plata+)</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>365</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Plata+; base terms 7-8%</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>https://www.rendimientosmexico.com/instrumentos/plata</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Openbank</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Apartados Open</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F129" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>Open+ debit account; 6.5% above 1M</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/openbank</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>conflict (see institutions)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>On demand (no Meli+)</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F130" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Without subscription</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/institucion/mercadopago</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>DiDi</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F131" t="n">
+        <v>10000</v>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Rate on balance above 10,000 not found</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>yes (excess rate unverified)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.0725</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>https://deceroalinfinito.com/mejores-sofipos</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Fixed term 30d</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>30</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.07049999999999999</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Fixed term 90d</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>90</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Fixed term 180d</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>180</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Stori</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Fixed term 365d</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>365</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.0825</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>On demand</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.0701</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>https://deceroalinfinito.com/mejores-sofipos</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Fixed term 30d</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>30</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Fixed term 90d</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>90</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Fixed term 180d</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>180</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.0759</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Finsus</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Fixed term 365d</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>365</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.08690000000000001</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Fixed term 90d</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>90</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Withdrawal problems reported May-Jun 2026</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Kubo Financiero</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Fixed term 365d</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>365</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Withdrawal problems reported May-Jun 2026</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
         <is>
           <t>CETES (via GBM or Cetesdirecto)</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CETES 28d</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>28</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.0615</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>CETES (via GBM or Cetesdirecto)</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>CETES 91d</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>91</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.0659</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>CETES (via GBM or Cetesdirecto)</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>CETES 182d</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>182</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.06909999999999999</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>https://www.tasas.mx/</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>CETES (via GBM or Cetesdirecto)</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
         <is>
           <t>CETES 364d</t>
         </is>
       </c>
-      <c r="D97" t="n">
+      <c r="D147" t="n">
         <v>364</v>
       </c>
-      <c r="E97" t="n">
+      <c r="E147" t="n">
         <v>0.07240000000000001</v>
       </c>
-      <c r="I97" t="inlineStr">
+      <c r="I147" t="inlineStr">
         <is>
           <t>https://www.tasas.mx/</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="J147" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
+      <c r="K147" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -34338,7 +36447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34434,7 +36543,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Previous year's rate, for comparison.</t>
+          <t>Previous year's rate, for comparison. Also stated in the Dec 2025 video (-rDq0PLHGs4).</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -34451,211 +36560,216 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>uma_daily_2026</t>
+          <t>isr_withholding_rate_2020</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>117.31</v>
+        <v>0.0145</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MXN</t>
+          <t>annual rate on invested capital</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>INEGI, DOF 2026-01-09.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/uma/uma2026.pdf</t>
+          <t>History only. Matches the Ley de Ingresos rate; no video found for it.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>not verified in videos</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>uma_annual_2026</t>
+          <t>isr_withholding_rate_2021</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42794.64</v>
+        <v>0.0097</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MXN</t>
+          <t>annual rate on invested capital</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>117.31 x 365 (rounded as published).</t>
+          <t>History only.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/uma/uma2026.pdf</t>
+          <t>https://www.youtube.com/watch?v=RcEoeHDvND8</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sofipo_exempt_limit_mxn</t>
+          <t>isr_withholding_rate_2022</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>213973.2</v>
+        <v>0.0008</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MXN average daily balance</t>
+          <t>annual rate on invested capital</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LISR art. 93 fr. XX: SOFIPO interest exempt if the average daily balance across all SOFIPOs is at most 5 annual UMAs; above it, only the excess is taxed.</t>
+          <t>History only. Big cut from 2021.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://es-us.noticias.yahoo.com/sofipos-impuestos-2026-cu%C3%A1nto-te-170000926.html</t>
+          <t>https://www.youtube.com/watch?v=RcEoeHDvND8</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>yes (secondary; statute not fetched directly)</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>bank_savings_exemption</t>
+          <t>isr_withholding_rate_2023</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0.0015</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>annual rate on invested capital</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Art. 93 fr. XX also exempts interest from bank savings/deposit accounts up to the same 5 UMAs (not fixed terms). Whether a bank applies it varies; the Sep 2026 video says Nu's Cajita Turbo is not withheld while Nu fixed terms are. Other banks' on-demand accounts are marked 'unknown' and taxed in the model.</t>
+          <t>History only.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.contadigital.mx/posts/isr-sobre-intereses-personas-fisicas</t>
+          <t>https://www.youtube.com/watch?v=fn7DOZ3qKQ0</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>secondary + video</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>udi_value</t>
+          <t>isr_withholding_rate_2024</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8.823864</v>
+        <v>0.005</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MXN per UDI</t>
+          <t>annual rate on invested capital</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Changes daily with inflation.</t>
+          <t>History only. 1.48% was proposed first (https://www.youtube.com/watch?v=00F_xLy5eRk).</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://calculadora-udi.com/</t>
+          <t>https://www.youtube.com/watch?v=Y9y3h_eOuGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>video (auto-captions)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>prosofipo_limit_udis</t>
+          <t>uma_daily_2026</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25000</v>
+        <v>117.31</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>UDIs</t>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Per person, per SOFIPO.</t>
+          <t>INEGI, DOF 2026-01-09.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/cnbv/articulos/seguros-de-deposito-que-protegen-tus-ahorros-en-instituciones-reguladas-y-supervisadas-por-cnbv?idiom=es</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/uma/uma2026.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>yes (secondary)</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>prosofipo_limit_mxn</t>
+          <t>uma_annual_2026</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>220596.6</v>
+        <v>42794.64</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -34664,85 +36778,250 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>25,000 x UDI value.</t>
+          <t>117.31 x 365 (rounded as published).</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://calculadora-udi.com/</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/uma/uma2026.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>computed</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ipab_limit_udis</t>
+          <t>sofipo_exempt_limit_mxn</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>400000</v>
+        <v>213973.2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>UDIs</t>
+          <t>MXN average daily balance</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Per person, per bank.</t>
+          <t>LISR art. 93 fr. XX: SOFIPO interest exempt if the average daily balance across all SOFIPOs is at most 5 annual UMAs; above it, only the excess is taxed.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.gob.mx/cnbv/articulos/seguros-de-deposito-que-protegen-tus-ahorros-en-instituciones-reguladas-y-supervisadas-por-cnbv?idiom=es</t>
+          <t>https://es-us.noticias.yahoo.com/sofipos-impuestos-2026-cu%C3%A1nto-te-170000926.html</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>yes (secondary)</t>
+          <t>yes (secondary; statute not fetched directly)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>bank_savings_exemption</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>flag</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Art. 93 fr. XX also exempts interest from bank savings/deposit accounts up to the same 5 UMAs (not fixed terms). Whether a bank applies it varies; the Sep 2026 video says Nu's Cajita Turbo is not withheld while Nu fixed terms are. Other banks' on-demand accounts are marked 'unknown' and taxed in the model.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.contadigital.mx/posts/isr-sobre-intereses-personas-fisicas</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>secondary + video</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>udi_value</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>8.823864</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MXN per UDI</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Changes daily with inflation.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://calculadora-udi.com/</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>prosofipo_limit_udis</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>25000</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>UDIs</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Per person, per SOFIPO.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://www.gob.mx/cnbv/articulos/seguros-de-deposito-que-protegen-tus-ahorros-en-instituciones-reguladas-y-supervisadas-por-cnbv?idiom=es</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>yes (secondary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>prosofipo_limit_mxn</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>220596.6</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MXN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>25,000 x UDI value.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://calculadora-udi.com/</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ipab_limit_udis</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>400000</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>UDIs</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Per person, per bank.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://www.gob.mx/cnbv/articulos/seguros-de-deposito-que-protegen-tus-ahorros-en-instituciones-reguladas-y-supervisadas-por-cnbv?idiom=es</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>yes (secondary)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>ipab_limit_mxn</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B17" t="n">
         <v>3529545.6</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>MXN</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>400,000 x UDI value.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://calculadora-udi.com/</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>computed</t>
         </is>

</xml_diff>